<commit_message>
Add data quality rules framework with 119 SQL rules
- dq framework: rule catalogue, run history, issue register, helper
  functions, and scorecard / detection views
- 119 rules (one view each) across master data, ERP, business Excel,
  SharePoint, and external data, with fix / quarantine / flag actions
- run_dq.py deploys and runs the rules and scores them against the
  generators' answer keys: 99.8% recall, 99.9% precision
- Fix generator bug where ws.cell(r, c, None) left planted blank
  safety stocks unchanged; regenerate business files (golden unchanged)
- Document rules, results, misses, and SQL Server pitfalls; record
  detection result in the duplicate supplier case study

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Source_Data/business_files/raw/excel/Safety_Stock_Targets_FY2026_FINAL.xlsx
+++ b/03_Source_Data/business_files/raw/excel/Safety_Stock_Targets_FY2026_FINAL.xlsx
@@ -3160,9 +3160,6 @@
           <t>4G-8533</t>
         </is>
       </c>
-      <c r="C116" t="n">
-        <v>2</v>
-      </c>
       <c r="D116" t="n">
         <v>3</v>
       </c>
@@ -5478,9 +5475,6 @@
           <t>138-4784</t>
         </is>
       </c>
-      <c r="C215" t="n">
-        <v>2</v>
-      </c>
       <c r="D215" t="n">
         <v>3</v>
       </c>
@@ -7360,9 +7354,6 @@
           <t>160-5817</t>
         </is>
       </c>
-      <c r="C295" t="n">
-        <v>2</v>
-      </c>
       <c r="D295" t="n">
         <v>3</v>
       </c>
@@ -8775,9 +8766,6 @@
         <is>
           <t>9L-6881</t>
         </is>
-      </c>
-      <c r="C354" t="n">
-        <v>2</v>
       </c>
       <c r="D354" t="n">
         <v>3</v>
@@ -16944,9 +16932,6 @@
         <is>
           <t>9P-3656</t>
         </is>
-      </c>
-      <c r="C277" t="n">
-        <v>2</v>
       </c>
       <c r="D277" t="n">
         <v>3</v>
@@ -22723,9 +22708,6 @@
           <t>9P-8996</t>
         </is>
       </c>
-      <c r="C128" t="n">
-        <v>3</v>
-      </c>
       <c r="D128" t="n">
         <v>4</v>
       </c>
@@ -25109,9 +25091,6 @@
           <t>448-1152</t>
         </is>
       </c>
-      <c r="C48" t="n">
-        <v>5</v>
-      </c>
       <c r="D48" t="n">
         <v>6</v>
       </c>
@@ -25876,9 +25855,6 @@
         <is>
           <t>8F-9785</t>
         </is>
-      </c>
-      <c r="C80" t="n">
-        <v>2</v>
       </c>
       <c r="D80" t="n">
         <v>3</v>
@@ -26577,9 +26553,6 @@
           <t>313-7717</t>
         </is>
       </c>
-      <c r="C110" t="n">
-        <v>3</v>
-      </c>
       <c r="D110" t="n">
         <v>4</v>
       </c>
@@ -27154,9 +27127,6 @@
         <is>
           <t>5J-4540</t>
         </is>
-      </c>
-      <c r="C134" t="n">
-        <v>3</v>
       </c>
       <c r="D134" t="n">
         <v>4</v>
@@ -31222,9 +31192,6 @@
           <t>4S-5275</t>
         </is>
       </c>
-      <c r="C306" t="n">
-        <v>23</v>
-      </c>
       <c r="D306" t="n">
         <v>24</v>
       </c>
@@ -31573,9 +31540,6 @@
           <t>1M-1092</t>
         </is>
       </c>
-      <c r="C322" t="n">
-        <v>4</v>
-      </c>
       <c r="D322" t="n">
         <v>5</v>
       </c>
@@ -32634,9 +32598,6 @@
         <is>
           <t>524-2290</t>
         </is>
-      </c>
-      <c r="C366" t="n">
-        <v>11</v>
       </c>
       <c r="D366" t="n">
         <v>16</v>
@@ -33644,9 +33605,6 @@
           <t>1B-5868</t>
         </is>
       </c>
-      <c r="C409" t="n">
-        <v>9</v>
-      </c>
       <c r="D409" t="n">
         <v>13</v>
       </c>
@@ -36498,9 +36456,6 @@
         <is>
           <t>480-8325</t>
         </is>
-      </c>
-      <c r="C529" t="n">
-        <v>4</v>
       </c>
       <c r="D529" t="n">
         <v>5</v>

</xml_diff>